<commit_message>
[DX12] Finalize recipe randomization
</commit_message>
<xml_diff>
--- a/docs/Items.xlsx
+++ b/docs/Items.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\RE_Modding\BioRand\re7\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC687770-2D01-44DC-A64D-2A7242C2C943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A360A7-BD33-4A23-9CD3-3A847A46CEC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2220" windowWidth="29040" windowHeight="15720" xr2:uid="{DE583D23-C62C-4A13-9B57-9882812AC707}"/>
+    <workbookView xWindow="38400" yWindow="2580" windowWidth="28800" windowHeight="15345" xr2:uid="{DE583D23-C62C-4A13-9B57-9882812AC707}"/>
   </bookViews>
   <sheets>
     <sheet name="items" sheetId="2" r:id="rId1"/>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">items!$A$1:$N$314</definedName>
@@ -2626,17 +2625,18 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8997F09E-7585-4546-A99D-93C95A83DDE6}" name="items" displayName="items" ref="A1:N314" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:N314" xr:uid="{8997F09E-7585-4546-A99D-93C95A83DDE6}">
-    <filterColumn colId="2">
+    <filterColumn colId="3">
       <filters>
-        <filter val="Drug"/>
-        <filter val="Material"/>
-        <filter val="Shell"/>
+        <filter val="Slot1"/>
       </filters>
     </filterColumn>
-    <filterColumn colId="13">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="WAHR"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="5">
+      <filters blank="1"/>
     </filterColumn>
   </autoFilter>
   <tableColumns count="14">
@@ -3215,7 +3215,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -3391,7 +3391,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -4007,7 +4007,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>83</v>
       </c>
@@ -4051,7 +4051,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>86</v>
       </c>
@@ -4227,7 +4227,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>95</v>
       </c>
@@ -4975,7 +4975,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>134</v>
       </c>
@@ -5019,7 +5019,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>137</v>
       </c>
@@ -5063,7 +5063,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>140</v>
       </c>
@@ -5107,7 +5107,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="49" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>143</v>
       </c>
@@ -5371,7 +5371,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="55" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>159</v>
       </c>
@@ -5635,7 +5635,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>174</v>
       </c>
@@ -6691,7 +6691,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="85" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>242</v>
       </c>
@@ -7307,7 +7307,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>276</v>
       </c>
@@ -7351,7 +7351,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>279</v>
       </c>
@@ -9683,7 +9683,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>429</v>
       </c>
@@ -9859,7 +9859,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="157" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>437</v>
       </c>
@@ -10035,7 +10035,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>445</v>
       </c>
@@ -10079,7 +10079,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>447</v>
       </c>
@@ -10167,7 +10167,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>451</v>
       </c>
@@ -10871,7 +10871,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="180" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>485</v>
       </c>
@@ -11003,7 +11003,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="183" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>492</v>
       </c>
@@ -12059,7 +12059,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="207" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>553</v>
       </c>
@@ -12103,7 +12103,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="208" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>555</v>
       </c>
@@ -12895,7 +12895,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="226" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>599</v>
       </c>
@@ -15931,7 +15931,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="295" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>752</v>
       </c>
@@ -16679,7 +16679,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="312" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>797</v>
       </c>
@@ -16816,15 +16816,6 @@
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9824B75-038E-4818-8E8A-41D34C263D5F}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Begin implementation of starting inventory randomization
</commit_message>
<xml_diff>
--- a/docs/Items.xlsx
+++ b/docs/Items.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\RE_Modding\BioRand\re7\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A360A7-BD33-4A23-9CD3-3A847A46CEC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8006D013-8FF4-4C1E-A943-0F46613589FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="2580" windowWidth="28800" windowHeight="15345" xr2:uid="{DE583D23-C62C-4A13-9B57-9882812AC707}"/>
+    <workbookView xWindow="38280" yWindow="2220" windowWidth="29040" windowHeight="15720" xr2:uid="{DE583D23-C62C-4A13-9B57-9882812AC707}"/>
   </bookViews>
   <sheets>
     <sheet name="items" sheetId="2" r:id="rId1"/>
@@ -2625,16 +2625,6 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8997F09E-7585-4546-A99D-93C95A83DDE6}" name="items" displayName="items" ref="A1:N314" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:N314" xr:uid="{8997F09E-7585-4546-A99D-93C95A83DDE6}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="Slot1"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="4">
-      <filters>
-        <filter val="WAHR"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="5">
       <filters blank="1"/>
     </filterColumn>
@@ -3039,7 +3029,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -3083,7 +3073,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -3171,7 +3161,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -3215,7 +3205,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -3259,7 +3249,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -3347,7 +3337,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -3435,7 +3425,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>46</v>
       </c>
@@ -3479,7 +3469,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>48</v>
       </c>
@@ -3523,7 +3513,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>51</v>
       </c>
@@ -3567,7 +3557,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>54</v>
       </c>
@@ -4095,7 +4085,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>89</v>
       </c>
@@ -4139,7 +4129,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="27" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>91</v>
       </c>
@@ -4183,7 +4173,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>94</v>
       </c>
@@ -4227,7 +4217,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="29" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>95</v>
       </c>
@@ -4271,7 +4261,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="30" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>97</v>
       </c>
@@ -4315,7 +4305,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="31" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>99</v>
       </c>
@@ -4359,7 +4349,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="32" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>101</v>
       </c>
@@ -4403,7 +4393,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>104</v>
       </c>
@@ -4447,7 +4437,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="34" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>105</v>
       </c>
@@ -4535,7 +4525,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>109</v>
       </c>
@@ -4579,7 +4569,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="37" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>111</v>
       </c>
@@ -4623,7 +4613,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="38" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>113</v>
       </c>
@@ -4667,7 +4657,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="39" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>115</v>
       </c>
@@ -4711,7 +4701,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="40" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>118</v>
       </c>
@@ -4755,7 +4745,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="41" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>121</v>
       </c>
@@ -4799,7 +4789,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="42" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>123</v>
       </c>
@@ -4843,7 +4833,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="43" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>125</v>
       </c>
@@ -4887,7 +4877,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="44" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>128</v>
       </c>
@@ -4931,7 +4921,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>131</v>
       </c>
@@ -4975,7 +4965,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>134</v>
       </c>
@@ -5019,7 +5009,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="47" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>137</v>
       </c>
@@ -5063,7 +5053,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="48" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>140</v>
       </c>
@@ -5151,7 +5141,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="50" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>145</v>
       </c>
@@ -5327,7 +5317,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="54" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>155</v>
       </c>
@@ -5459,7 +5449,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="57" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>165</v>
       </c>
@@ -5547,7 +5537,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="59" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>169</v>
       </c>
@@ -5635,7 +5625,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="61" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>174</v>
       </c>
@@ -6603,7 +6593,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="83" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>236</v>
       </c>
@@ -6647,7 +6637,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="84" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>239</v>
       </c>
@@ -6779,7 +6769,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="87" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>248</v>
       </c>
@@ -6867,7 +6857,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>252</v>
       </c>
@@ -6911,7 +6901,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="90" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>254</v>
       </c>
@@ -6955,7 +6945,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="91" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>257</v>
       </c>
@@ -6999,7 +6989,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="92" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>260</v>
       </c>
@@ -7043,7 +7033,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="93" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>262</v>
       </c>
@@ -7087,7 +7077,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="94" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>265</v>
       </c>
@@ -7131,7 +7121,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="95" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>267</v>
       </c>
@@ -7175,7 +7165,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="96" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>269</v>
       </c>
@@ -7219,7 +7209,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="97" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>271</v>
       </c>
@@ -7307,7 +7297,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="99" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>276</v>
       </c>
@@ -7351,7 +7341,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="100" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>279</v>
       </c>
@@ -7395,7 +7385,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="101" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>281</v>
       </c>
@@ -7439,7 +7429,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="102" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>284</v>
       </c>
@@ -8319,7 +8309,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="122" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>344</v>
       </c>
@@ -8363,7 +8353,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="123" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>346</v>
       </c>
@@ -8407,7 +8397,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="124" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>348</v>
       </c>
@@ -8451,7 +8441,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="125" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>350</v>
       </c>
@@ -8495,7 +8485,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="126" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>353</v>
       </c>
@@ -8539,7 +8529,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="127" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>354</v>
       </c>
@@ -9023,7 +9013,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="138" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>385</v>
       </c>
@@ -9067,7 +9057,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="139" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>388</v>
       </c>
@@ -9111,7 +9101,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="140" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>391</v>
       </c>
@@ -9639,7 +9629,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="152" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>427</v>
       </c>
@@ -9683,7 +9673,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="153" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>429</v>
       </c>
@@ -9727,7 +9717,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="154" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>431</v>
       </c>
@@ -9771,7 +9761,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="155" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>433</v>
       </c>
@@ -9815,7 +9805,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="156" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>435</v>
       </c>
@@ -9903,7 +9893,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="158" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>439</v>
       </c>
@@ -9947,7 +9937,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="159" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>441</v>
       </c>
@@ -9991,7 +9981,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="160" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>443</v>
       </c>
@@ -10035,7 +10025,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="161" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>445</v>
       </c>
@@ -10079,7 +10069,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="162" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>447</v>
       </c>
@@ -10167,7 +10157,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="164" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>451</v>
       </c>
@@ -10343,7 +10333,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="168" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>366</v>
       </c>
@@ -10387,7 +10377,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="169" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>459</v>
       </c>
@@ -10695,7 +10685,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="176" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>474</v>
       </c>
@@ -10739,7 +10729,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="177" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>477</v>
       </c>
@@ -10783,7 +10773,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="178" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>480</v>
       </c>
@@ -10827,7 +10817,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="179" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>483</v>
       </c>
@@ -10871,7 +10861,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="180" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>485</v>
       </c>
@@ -10915,7 +10905,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="181" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>487</v>
       </c>
@@ -10959,7 +10949,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="182" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>490</v>
       </c>
@@ -11003,7 +10993,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="183" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>492</v>
       </c>
@@ -11047,7 +11037,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="184" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>494</v>
       </c>
@@ -11091,7 +11081,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="185" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>117</v>
       </c>
@@ -11135,7 +11125,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="186" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>498</v>
       </c>
@@ -11179,7 +11169,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="187" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>501</v>
       </c>
@@ -11223,7 +11213,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="188" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>503</v>
       </c>
@@ -11399,7 +11389,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="192" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>513</v>
       </c>
@@ -11487,7 +11477,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="194" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>517</v>
       </c>
@@ -11531,7 +11521,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="195" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>520</v>
       </c>
@@ -11795,7 +11785,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="201" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>538</v>
       </c>
@@ -11839,7 +11829,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="202" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>541</v>
       </c>
@@ -11883,7 +11873,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="203" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>544</v>
       </c>
@@ -11927,7 +11917,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="204" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>547</v>
       </c>
@@ -11971,7 +11961,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="205" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>549</v>
       </c>
@@ -12059,7 +12049,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="207" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>553</v>
       </c>
@@ -12103,7 +12093,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="208" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>555</v>
       </c>
@@ -12191,7 +12181,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="210" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>559</v>
       </c>
@@ -12411,7 +12401,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="215" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>572</v>
       </c>
@@ -12455,7 +12445,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="216" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>575</v>
       </c>
@@ -12499,7 +12489,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="217" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>577</v>
       </c>
@@ -12543,7 +12533,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="218" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>579</v>
       </c>
@@ -12587,7 +12577,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="219" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>581</v>
       </c>
@@ -12631,7 +12621,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="220" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>583</v>
       </c>
@@ -12807,7 +12797,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="224" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>595</v>
       </c>
@@ -12851,7 +12841,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="225" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>597</v>
       </c>
@@ -12895,7 +12885,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="226" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>599</v>
       </c>
@@ -12939,7 +12929,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="227" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>601</v>
       </c>
@@ -12983,7 +12973,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="228" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>603</v>
       </c>
@@ -13027,7 +13017,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="229" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>606</v>
       </c>
@@ -13071,7 +13061,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="230" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>609</v>
       </c>
@@ -15183,7 +15173,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="278" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>705</v>
       </c>
@@ -15315,7 +15305,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="281" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>713</v>
       </c>
@@ -15931,7 +15921,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="295" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>752</v>
       </c>
@@ -15975,7 +15965,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="296" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>754</v>
       </c>
@@ -16019,7 +16009,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="297" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>757</v>
       </c>
@@ -16063,7 +16053,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="298" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>759</v>
       </c>
@@ -16107,7 +16097,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="299" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>762</v>
       </c>
@@ -16503,7 +16493,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="308" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>787</v>
       </c>
@@ -16547,7 +16537,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="309" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>790</v>
       </c>
@@ -16591,7 +16581,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="310" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>792</v>
       </c>
@@ -16723,7 +16713,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="313" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>799</v>
       </c>
@@ -16767,7 +16757,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="314" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>801</v>
       </c>

</xml_diff>

<commit_message>
Define story progression items
</commit_message>
<xml_diff>
--- a/docs/Items.xlsx
+++ b/docs/Items.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\RE_Modding\BioRand\re7\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A29A7605-01F8-41DB-BFD0-F7A0F507BA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32BA5522-0AB6-4704-AD28-C73EEC8F74DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2220" windowWidth="29040" windowHeight="15720" xr2:uid="{DE583D23-C62C-4A13-9B57-9882812AC707}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DE583D23-C62C-4A13-9B57-9882812AC707}"/>
   </bookViews>
   <sheets>
     <sheet name="items" sheetId="2" r:id="rId1"/>
@@ -2624,11 +2624,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8997F09E-7585-4546-A99D-93C95A83DDE6}" name="items" displayName="items" ref="A1:N314" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:N314" xr:uid="{8997F09E-7585-4546-A99D-93C95A83DDE6}">
-    <filterColumn colId="5">
-      <filters blank="1"/>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:N314" xr:uid="{8997F09E-7585-4546-A99D-93C95A83DDE6}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{F0F4938D-6AE6-4FD1-903A-6D70073C8CFE}" uniqueName="1" name="Id" queryTableFieldId="1" dataDxfId="12"/>
     <tableColumn id="2" xr3:uid="{0EDD0777-3DC7-4A87-90CA-8CAF0D26BB97}" uniqueName="2" name="Name" queryTableFieldId="2" dataDxfId="11"/>
@@ -3117,7 +3113,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -3293,7 +3289,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -3601,7 +3597,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>55</v>
       </c>
@@ -3645,7 +3641,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>60</v>
       </c>
@@ -3689,7 +3685,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>63</v>
       </c>
@@ -3733,7 +3729,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>66</v>
       </c>
@@ -3777,7 +3773,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>69</v>
       </c>
@@ -3821,7 +3817,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>72</v>
       </c>
@@ -3865,7 +3861,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>74</v>
       </c>
@@ -3909,7 +3905,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -3953,7 +3949,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>80</v>
       </c>
@@ -4481,7 +4477,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="35" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>106</v>
       </c>
@@ -5185,7 +5181,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="51" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>146</v>
       </c>
@@ -5229,7 +5225,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>149</v>
       </c>
@@ -5273,7 +5269,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>152</v>
       </c>
@@ -5405,7 +5401,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>162</v>
       </c>
@@ -5493,7 +5489,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>167</v>
       </c>
@@ -5581,7 +5577,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="60" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>171</v>
       </c>
@@ -5669,7 +5665,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="62" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>177</v>
       </c>
@@ -5713,7 +5709,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="63" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>179</v>
       </c>
@@ -5757,7 +5753,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="64" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>182</v>
       </c>
@@ -5801,7 +5797,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="65" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>184</v>
       </c>
@@ -5845,7 +5841,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>186</v>
       </c>
@@ -5889,7 +5885,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>189</v>
       </c>
@@ -5933,7 +5929,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="68" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>192</v>
       </c>
@@ -5977,7 +5973,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="69" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>194</v>
       </c>
@@ -6021,7 +6017,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="70" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>196</v>
       </c>
@@ -6065,7 +6061,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="71" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>200</v>
       </c>
@@ -6109,7 +6105,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="72" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>203</v>
       </c>
@@ -6153,7 +6149,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="73" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>206</v>
       </c>
@@ -6197,7 +6193,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="74" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>209</v>
       </c>
@@ -6241,7 +6237,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>212</v>
       </c>
@@ -6285,7 +6281,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="76" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>215</v>
       </c>
@@ -6329,7 +6325,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="77" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>218</v>
       </c>
@@ -6373,7 +6369,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="78" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>221</v>
       </c>
@@ -6417,7 +6413,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="79" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>224</v>
       </c>
@@ -6461,7 +6457,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="80" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>227</v>
       </c>
@@ -6505,7 +6501,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="81" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>230</v>
       </c>
@@ -6549,7 +6545,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="82" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>233</v>
       </c>
@@ -6725,7 +6721,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="86" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>245</v>
       </c>
@@ -6813,7 +6809,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="88" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>250</v>
       </c>
@@ -7253,7 +7249,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="98" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>274</v>
       </c>
@@ -7473,7 +7469,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="103" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>287</v>
       </c>
@@ -7517,7 +7513,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="104" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>290</v>
       </c>
@@ -7561,7 +7557,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="105" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>293</v>
       </c>
@@ -7605,7 +7601,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="106" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>296</v>
       </c>
@@ -7649,7 +7645,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="107" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>299</v>
       </c>
@@ -7693,7 +7689,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="108" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>302</v>
       </c>
@@ -7737,7 +7733,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="109" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>305</v>
       </c>
@@ -7781,7 +7777,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="110" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>308</v>
       </c>
@@ -7825,7 +7821,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="111" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>311</v>
       </c>
@@ -7869,7 +7865,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="112" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>314</v>
       </c>
@@ -7913,7 +7909,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="113" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>317</v>
       </c>
@@ -7957,7 +7953,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="114" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>320</v>
       </c>
@@ -8001,7 +7997,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="115" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>323</v>
       </c>
@@ -8045,7 +8041,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="116" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>326</v>
       </c>
@@ -8089,7 +8085,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="117" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>329</v>
       </c>
@@ -8133,7 +8129,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="118" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>332</v>
       </c>
@@ -8177,7 +8173,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="119" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>335</v>
       </c>
@@ -8221,7 +8217,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="120" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>338</v>
       </c>
@@ -8265,7 +8261,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="121" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>341</v>
       </c>
@@ -8573,7 +8569,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="128" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>357</v>
       </c>
@@ -8617,7 +8613,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="129" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>360</v>
       </c>
@@ -8661,7 +8657,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="130" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>363</v>
       </c>
@@ -8705,7 +8701,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="131" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>365</v>
       </c>
@@ -8749,7 +8745,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="132" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>367</v>
       </c>
@@ -8793,7 +8789,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="133" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>370</v>
       </c>
@@ -8837,7 +8833,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="134" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>373</v>
       </c>
@@ -8881,7 +8877,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="135" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>376</v>
       </c>
@@ -8925,7 +8921,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="136" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>379</v>
       </c>
@@ -8969,7 +8965,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="137" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>382</v>
       </c>
@@ -9145,7 +9141,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="141" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>392</v>
       </c>
@@ -9189,7 +9185,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="142" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>395</v>
       </c>
@@ -9233,7 +9229,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="143" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>398</v>
       </c>
@@ -9277,7 +9273,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="144" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>401</v>
       </c>
@@ -9321,7 +9317,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="145" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>403</v>
       </c>
@@ -9365,7 +9361,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="146" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>404</v>
       </c>
@@ -9409,7 +9405,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="147" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>408</v>
       </c>
@@ -9453,7 +9449,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="148" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>412</v>
       </c>
@@ -9497,7 +9493,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="149" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>416</v>
       </c>
@@ -9541,7 +9537,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="150" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>420</v>
       </c>
@@ -9585,7 +9581,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="151" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>424</v>
       </c>
@@ -10113,7 +10109,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="163" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>449</v>
       </c>
@@ -10201,7 +10197,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="165" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>453</v>
       </c>
@@ -10245,7 +10241,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="166" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>455</v>
       </c>
@@ -10289,7 +10285,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="167" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>456</v>
       </c>
@@ -10421,7 +10417,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="170" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>461</v>
       </c>
@@ -10465,7 +10461,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="171" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>462</v>
       </c>
@@ -10509,7 +10505,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="172" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>465</v>
       </c>
@@ -10553,7 +10549,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="173" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>468</v>
       </c>
@@ -10597,7 +10593,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="174" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>471</v>
       </c>
@@ -10641,7 +10637,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="175" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>472</v>
       </c>
@@ -11257,7 +11253,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="189" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>505</v>
       </c>
@@ -11301,7 +11297,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="190" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>507</v>
       </c>
@@ -11345,7 +11341,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="191" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>510</v>
       </c>
@@ -11433,7 +11429,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="193" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>515</v>
       </c>
@@ -11565,7 +11561,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="196" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>523</v>
       </c>
@@ -11609,7 +11605,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="197" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>526</v>
       </c>
@@ -11653,7 +11649,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="198" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>529</v>
       </c>
@@ -11697,7 +11693,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="199" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>532</v>
       </c>
@@ -11741,7 +11737,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="200" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>535</v>
       </c>
@@ -12005,7 +12001,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="206" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>551</v>
       </c>
@@ -12137,7 +12133,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="209" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>557</v>
       </c>
@@ -12225,7 +12221,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="211" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>562</v>
       </c>
@@ -12269,7 +12265,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="212" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>565</v>
       </c>
@@ -12313,7 +12309,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="213" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>567</v>
       </c>
@@ -12357,7 +12353,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="214" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>569</v>
       </c>
@@ -12665,7 +12661,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="221" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>586</v>
       </c>
@@ -12709,7 +12705,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="222" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>589</v>
       </c>
@@ -12753,7 +12749,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="223" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>592</v>
       </c>
@@ -13105,7 +13101,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="231" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>611</v>
       </c>
@@ -13149,7 +13145,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="232" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>614</v>
       </c>
@@ -13193,7 +13189,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="233" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>615</v>
       </c>
@@ -13237,7 +13233,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="234" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>618</v>
       </c>
@@ -13281,7 +13277,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="235" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>619</v>
       </c>
@@ -13325,7 +13321,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="236" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>622</v>
       </c>
@@ -13369,7 +13365,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="237" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>623</v>
       </c>
@@ -13413,7 +13409,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="238" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>626</v>
       </c>
@@ -13457,7 +13453,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="239" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>627</v>
       </c>
@@ -13501,7 +13497,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="240" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>630</v>
       </c>
@@ -13545,7 +13541,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="241" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>631</v>
       </c>
@@ -13589,7 +13585,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="242" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>634</v>
       </c>
@@ -13633,7 +13629,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="243" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>635</v>
       </c>
@@ -13677,7 +13673,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="244" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>638</v>
       </c>
@@ -13721,7 +13717,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="245" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>639</v>
       </c>
@@ -13765,7 +13761,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="246" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>642</v>
       </c>
@@ -13809,7 +13805,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="247" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>643</v>
       </c>
@@ -13853,7 +13849,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="248" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>646</v>
       </c>
@@ -13897,7 +13893,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="249" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>647</v>
       </c>
@@ -13941,7 +13937,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="250" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>650</v>
       </c>
@@ -13985,7 +13981,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="251" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>651</v>
       </c>
@@ -14029,7 +14025,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="252" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>654</v>
       </c>
@@ -14073,7 +14069,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="253" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>655</v>
       </c>
@@ -14117,7 +14113,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="254" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>658</v>
       </c>
@@ -14161,7 +14157,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="255" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>659</v>
       </c>
@@ -14205,7 +14201,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="256" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>662</v>
       </c>
@@ -14249,7 +14245,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="257" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>663</v>
       </c>
@@ -14293,7 +14289,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="258" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>666</v>
       </c>
@@ -14337,7 +14333,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="259" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>667</v>
       </c>
@@ -14381,7 +14377,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="260" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>670</v>
       </c>
@@ -14425,7 +14421,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="261" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>671</v>
       </c>
@@ -14469,7 +14465,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="262" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>674</v>
       </c>
@@ -14513,7 +14509,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="263" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>675</v>
       </c>
@@ -14557,7 +14553,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="264" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>678</v>
       </c>
@@ -14601,7 +14597,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="265" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>679</v>
       </c>
@@ -14645,7 +14641,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="266" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>682</v>
       </c>
@@ -14689,7 +14685,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="267" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>683</v>
       </c>
@@ -14733,7 +14729,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="268" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>686</v>
       </c>
@@ -14777,7 +14773,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="269" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>687</v>
       </c>
@@ -14821,7 +14817,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="270" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>690</v>
       </c>
@@ -14865,7 +14861,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="271" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>691</v>
       </c>
@@ -14909,7 +14905,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="272" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>694</v>
       </c>
@@ -14953,7 +14949,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="273" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>695</v>
       </c>
@@ -14997,7 +14993,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="274" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>698</v>
       </c>
@@ -15041,7 +15037,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="275" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>699</v>
       </c>
@@ -15085,7 +15081,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="276" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>702</v>
       </c>
@@ -15129,7 +15125,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="277" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>703</v>
       </c>
@@ -15217,7 +15213,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="279" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>707</v>
       </c>
@@ -15261,7 +15257,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="280" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>710</v>
       </c>
@@ -15349,7 +15345,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="282" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>715</v>
       </c>
@@ -15393,7 +15389,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="283" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>717</v>
       </c>
@@ -15437,7 +15433,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="284" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>720</v>
       </c>
@@ -15481,7 +15477,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="285" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>723</v>
       </c>
@@ -15525,7 +15521,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="286" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>726</v>
       </c>
@@ -15569,7 +15565,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="287" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>729</v>
       </c>
@@ -15613,7 +15609,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="288" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>732</v>
       </c>
@@ -15657,7 +15653,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="289" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>735</v>
       </c>
@@ -15701,7 +15697,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="290" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>738</v>
       </c>
@@ -15745,7 +15741,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="291" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>741</v>
       </c>
@@ -15789,7 +15785,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="292" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>744</v>
       </c>
@@ -15833,7 +15829,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="293" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>746</v>
       </c>
@@ -15877,7 +15873,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="294" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>749</v>
       </c>
@@ -16141,7 +16137,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="300" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>764</v>
       </c>
@@ -16185,7 +16181,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="301" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>766</v>
       </c>
@@ -16229,7 +16225,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="302" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>769</v>
       </c>
@@ -16273,7 +16269,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="303" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>772</v>
       </c>
@@ -16317,7 +16313,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="304" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>775</v>
       </c>
@@ -16361,7 +16357,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="305" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>778</v>
       </c>
@@ -16405,7 +16401,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="306" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>781</v>
       </c>
@@ -16449,7 +16445,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="307" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>784</v>
       </c>
@@ -16625,7 +16621,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="311" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>794</v>
       </c>

</xml_diff>